<commit_message>
Saved progress at the end of the loop
Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 99972cae-3e15-4549-931f-339b8bc4b3e4
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 93b11ecb-1eaf-4ec4-b5b5-872c1a000107
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/2f8f6fb6-6daf-4be4-bbb0-0f1abd3223bf/99972cae-3e15-4549-931f-339b8bc4b3e4/ZvxUUP3
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/outputs/schedule_kenkere.xlsx
+++ b/outputs/schedule_kenkere.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Iteration 2" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Iteration 3" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Main" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Iteration 2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Iteration 3" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -983,9 +983,9 @@
 [CONSIDER]</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>FIT
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>Mat 57
 Pushyank Nahar
 38% pred | 0% hist
 [CONSIDER]</t>
@@ -1535,9 +1535,9 @@
 [CONSIDER]</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>FIT
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>Mat 57
 Pushyank Nahar
 38% pred | 0% hist
 [CONSIDER]</t>
@@ -2087,9 +2087,9 @@
 [CONSIDER]</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>FIT
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>Mat 57
 Pushyank Nahar
 38% pred | 0% hist
 [CONSIDER]</t>

</xml_diff>

<commit_message>
Update scheduling logic and disable unused rules for improved performance
Modify scoring algorithm in scorer.py to correctly use fill percentage, disable several rules in rules_config.json, and update output files and state data.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 99972cae-3e15-4549-931f-339b8bc4b3e4
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 423966cd-c064-42ab-8d50-516540e4b2a8
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/2f8f6fb6-6daf-4be4-bbb0-0f1abd3223bf/99972cae-3e15-4549-931f-339b8bc4b3e4/Week7bA
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/outputs/schedule_kenkere.xlsx
+++ b/outputs/schedule_kenkere.xlsx
@@ -810,12 +810,12 @@
 [PINNED]</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>Barre 57
-Shruti Kulkarni
-52% pred | 0% hist
-[PINNED]</t>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>Recovery
+Shruti Suresh
+38% pred | 0% hist
+[DROP]</t>
         </is>
       </c>
     </row>
@@ -836,7 +836,7 @@
           <t>Back Body Blaze
 Shruti Kulkarni
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
     </row>
@@ -863,7 +863,7 @@
           <t>FIT
 Pushyank Nahar
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="H10" s="6" t="n"/>
@@ -882,8 +882,8 @@
       <c r="G11" s="5" t="inlineStr">
         <is>
           <t>Cardio Barre
-Shruti Kulkarni
-17% pred | 17% hist
+Siddhartha Kusuma
+19% pred | 19% hist
 [CONSIDER]</t>
         </is>
       </c>
@@ -900,7 +900,7 @@
           <t>Mat 57
 Shruti Kulkarni
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
@@ -916,7 +916,7 @@
           <t>Mat 57
 Pushyank Nahar
 43% pred | 43% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -940,7 +940,7 @@
           <t>Mat 57
 Pushyank Nahar
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="H12" s="6" t="n"/>
@@ -988,7 +988,7 @@
           <t>Mat 57
 Pushyank Nahar
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
@@ -996,7 +996,7 @@
           <t>Recovery
 Shruti Kulkarni
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="H13" s="6" t="n"/>
@@ -1012,7 +1012,7 @@
           <t>Recovery
 Shruti Kulkarni
 10% pred | 10% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
@@ -1020,7 +1020,7 @@
           <t>Recovery
 Shruti Kulkarni
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -1028,7 +1028,7 @@
           <t>FIT
 Pushyank Nahar
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="E14" s="10" t="inlineStr">
@@ -1036,7 +1036,7 @@
           <t>Recovery
 Shruti Kulkarni
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -1063,7 +1063,7 @@
           <t>Back Body Blaze
 Shruti Kulkarni
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="E15" s="6" t="n"/>
@@ -1362,12 +1362,12 @@
 [PINNED]</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>Barre 57
-Shruti Kulkarni
-52% pred | 0% hist
-[PINNED]</t>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>Recovery
+Shruti Suresh
+38% pred | 0% hist
+[DROP]</t>
         </is>
       </c>
     </row>
@@ -1388,7 +1388,7 @@
           <t>Back Body Blaze
 Shruti Kulkarni
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
     </row>
@@ -1415,7 +1415,7 @@
           <t>FIT
 Pushyank Nahar
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="H10" s="6" t="n"/>
@@ -1434,8 +1434,8 @@
       <c r="G11" s="5" t="inlineStr">
         <is>
           <t>Cardio Barre
-Shruti Kulkarni
-17% pred | 17% hist
+Siddhartha Kusuma
+19% pred | 19% hist
 [CONSIDER]</t>
         </is>
       </c>
@@ -1452,7 +1452,7 @@
           <t>Mat 57
 Shruti Kulkarni
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
@@ -1468,7 +1468,7 @@
           <t>Mat 57
 Pushyank Nahar
 43% pred | 43% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -1492,7 +1492,7 @@
           <t>Mat 57
 Pushyank Nahar
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="H12" s="6" t="n"/>
@@ -1540,7 +1540,7 @@
           <t>Mat 57
 Pushyank Nahar
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
@@ -1548,7 +1548,7 @@
           <t>Recovery
 Shruti Kulkarni
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="H13" s="6" t="n"/>
@@ -1564,7 +1564,7 @@
           <t>Recovery
 Shruti Kulkarni
 10% pred | 10% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
@@ -1572,7 +1572,7 @@
           <t>Recovery
 Shruti Kulkarni
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -1580,7 +1580,7 @@
           <t>FIT
 Pushyank Nahar
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="E14" s="10" t="inlineStr">
@@ -1588,7 +1588,7 @@
           <t>Recovery
 Shruti Kulkarni
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -1615,7 +1615,7 @@
           <t>Back Body Blaze
 Shruti Kulkarni
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="E15" s="6" t="n"/>
@@ -1914,12 +1914,12 @@
 [PINNED]</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>Barre 57
-Shruti Kulkarni
-52% pred | 0% hist
-[PINNED]</t>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>Recovery
+Shruti Suresh
+38% pred | 0% hist
+[DROP]</t>
         </is>
       </c>
     </row>
@@ -1940,7 +1940,7 @@
           <t>Back Body Blaze
 Shruti Kulkarni
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
     </row>
@@ -1967,7 +1967,7 @@
           <t>FIT
 Pushyank Nahar
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="H10" s="6" t="n"/>
@@ -1986,8 +1986,8 @@
       <c r="G11" s="5" t="inlineStr">
         <is>
           <t>Cardio Barre
-Shruti Kulkarni
-17% pred | 17% hist
+Siddhartha Kusuma
+19% pred | 19% hist
 [CONSIDER]</t>
         </is>
       </c>
@@ -2004,7 +2004,7 @@
           <t>Mat 57
 Shruti Kulkarni
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
@@ -2020,7 +2020,7 @@
           <t>Mat 57
 Pushyank Nahar
 43% pred | 43% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2044,7 +2044,7 @@
           <t>Mat 57
 Pushyank Nahar
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="H12" s="6" t="n"/>
@@ -2092,7 +2092,7 @@
           <t>Mat 57
 Pushyank Nahar
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
@@ -2100,7 +2100,7 @@
           <t>Recovery
 Shruti Kulkarni
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="H13" s="6" t="n"/>
@@ -2116,7 +2116,7 @@
           <t>Recovery
 Shruti Kulkarni
 10% pred | 10% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
@@ -2124,7 +2124,7 @@
           <t>Recovery
 Shruti Kulkarni
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -2132,7 +2132,7 @@
           <t>FIT
 Pushyank Nahar
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="E14" s="10" t="inlineStr">
@@ -2140,7 +2140,7 @@
           <t>Recovery
 Shruti Kulkarni
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -2167,7 +2167,7 @@
           <t>Back Body Blaze
 Shruti Kulkarni
 38% pred | 0% hist
-[CONSIDER]</t>
+[PROTECT]</t>
         </is>
       </c>
       <c r="E15" s="6" t="n"/>

</xml_diff>

<commit_message>
Fix infinite loading on schedule generation and update output scores
Modify the API to return a status field for pipeline monitoring, and update generated schedules and scorecard data.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 99972cae-3e15-4549-931f-339b8bc4b3e4
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 07342bf3-9bb9-4fba-ba10-7a89658e0ca8
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/2f8f6fb6-6daf-4be4-bbb0-0f1abd3223bf/99972cae-3e15-4549-931f-339b8bc4b3e4/6JByfLg
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/outputs/schedule_kenkere.xlsx
+++ b/outputs/schedule_kenkere.xlsx
@@ -533,7 +533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -654,9 +654,9 @@
       <c r="C4" s="6" t="n"/>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Barre 57
-Siddhartha Kusuma
-0% pred | 0% hist
+          <t>Cardio Barre
+Shruti Kulkarni
+38% pred | 0% hist
 [CONSIDER]</t>
         </is>
       </c>
@@ -759,8 +759,8 @@
       <c r="C7" s="6" t="n"/>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Barre 57
-Siddhartha Kusuma
+          <t>Cardio Barre Plus
+Pushyank Nahar
 38% pred | 0% hist
 [CONSIDER]</t>
         </is>
@@ -768,7 +768,14 @@
       <c r="E7" s="6" t="n"/>
       <c r="F7" s="6" t="n"/>
       <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>FIT
+Siddhartha Kusuma
+38% pred | 0% hist
+[CONSIDER]</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="52" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
@@ -810,12 +817,12 @@
 [PINNED]</t>
         </is>
       </c>
-      <c r="H8" s="10" t="inlineStr">
-        <is>
-          <t>Recovery
-Shruti Suresh
-38% pred | 0% hist
-[DROP]</t>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Barre 57
+Shruti Kulkarni
+52% pred | 0% hist
+[PINNED]</t>
         </is>
       </c>
     </row>
@@ -851,7 +858,7 @@
       <c r="D10" s="6" t="n"/>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>FIT
+          <t>Back Body Blaze Express
 Shruti Kulkarni
 38% pred | 0% hist
 [DROP]</t>
@@ -869,22 +876,57 @@
       <c r="H10" s="6" t="n"/>
     </row>
     <row r="11" ht="52" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>17:15</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="n"/>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="n"/>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>FIT
+Shruti Kulkarni
+38% pred | 0% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Mat 57
+Shruti Kulkarni
+50% pred | 50% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Mat 57
+Shruti Kulkarni
+50% pred | 50% hist
+[PROTECT]</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Mat 57
+Shruti Kulkarni
+38% pred | 0% hist
+[PROTECT]</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>Cardio Barre
-Siddhartha Kusuma
-19% pred | 19% hist
-[CONSIDER]</t>
+Shruti Kulkarni
+38% pred | 0% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>Mat 57
+Pushyank Nahar
+38% pred | 0% hist
+[PROTECT]</t>
         </is>
       </c>
       <c r="H11" s="6" t="n"/>
@@ -892,55 +934,55 @@
     <row r="12" ht="52" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Mat 57
-Shruti Kulkarni
-38% pred | 0% hist
-[PROTECT]</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>Mat 57
-Shruti Kulkarni
-50% pred | 50% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>Mat 57
-Pushyank Nahar
-43% pred | 43% hist
-[PROTECT]</t>
-        </is>
-      </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t>Mat 57
-Shruti Kulkarni
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Barre 57
+Chaitanya Nahar
+19% pred | 19% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Barre 57
+Shruti Suresh
+38% pred | 0% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Barre 57
+Siddhartha Kusuma
+31% pred | 31% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Barre 57
+Shruti Suresh
 38% pred | 0% hist
 [CONSIDER]</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
+          <t>FIT
+Pushyank Nahar
+38% pred | 0% hist
+[PROTECT]</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
           <t>Cardio Barre
-Shruti Kulkarni
-38% pred | 0% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="G12" s="9" t="inlineStr">
-        <is>
-          <t>Mat 57
-Pushyank Nahar
-38% pred | 0% hist
-[PROTECT]</t>
+Chaitanya Nahar
+38% pred | 0% hist
+[CONSIDER]</t>
         </is>
       </c>
       <c r="H12" s="6" t="n"/>
@@ -948,53 +990,53 @@
     <row r="13" ht="52" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>18:15</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Mat 57
+Shruti Kulkarni
+38% pred | 0% hist
+[PROTECT]</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Recovery
+Shruti Kulkarni
+38% pred | 0% hist
+[PROTECT]</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Back Body Blaze
+Shruti Kulkarni
+38% pred | 0% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>FIT
+Shruti Kulkarni
+38% pred | 0% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>Cardio Barre
-Siddhartha Kusuma
-38% pred | 0% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Barre 57
-Shruti Suresh
-38% pred | 0% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Barre 57
-Siddhartha Kusuma
-31% pred | 31% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Barre 57
-Shruti Suresh
-38% pred | 0% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="F13" s="9" t="inlineStr">
-        <is>
-          <t>Mat 57
-Pushyank Nahar
-38% pred | 0% hist
-[PROTECT]</t>
+Pushyank Nahar
+26% pred | 26% hist
+[CONSIDER]</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
           <t>Recovery
-Shruti Kulkarni
+Pushyank Nahar
 38% pred | 0% hist
 [PROTECT]</t>
         </is>
@@ -1004,25 +1046,11 @@
     <row r="14" ht="52" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>19:15</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>Recovery
-Shruti Kulkarni
-10% pred | 10% hist
-[PROTECT]</t>
-        </is>
-      </c>
-      <c r="C14" s="10" t="inlineStr">
-        <is>
-          <t>Recovery
-Shruti Kulkarni
-38% pred | 0% hist
-[PROTECT]</t>
-        </is>
-      </c>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
       <c r="D14" s="5" t="inlineStr">
         <is>
           <t>FIT
@@ -1031,45 +1059,10 @@
 [PROTECT]</t>
         </is>
       </c>
-      <c r="E14" s="10" t="inlineStr">
-        <is>
-          <t>Recovery
-Shruti Kulkarni
-38% pred | 0% hist
-[PROTECT]</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>Cardio Barre
-Pushyank Nahar
-26% pred | 26% hist
-[CONSIDER]</t>
-        </is>
-      </c>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="n"/>
       <c r="H14" s="6" t="n"/>
-    </row>
-    <row r="15" ht="52" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>19:30</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="n"/>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Back Body Blaze
-Shruti Kulkarni
-38% pred | 0% hist
-[PROTECT]</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="n"/>
-      <c r="G15" s="6" t="n"/>
-      <c r="H15" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1085,7 +1078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1206,9 +1199,9 @@
       <c r="C4" s="6" t="n"/>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Barre 57
-Siddhartha Kusuma
-0% pred | 0% hist
+          <t>Cardio Barre
+Shruti Kulkarni
+38% pred | 0% hist
 [CONSIDER]</t>
         </is>
       </c>
@@ -1311,8 +1304,8 @@
       <c r="C7" s="6" t="n"/>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Barre 57
-Siddhartha Kusuma
+          <t>Cardio Barre Plus
+Pushyank Nahar
 38% pred | 0% hist
 [CONSIDER]</t>
         </is>
@@ -1320,7 +1313,14 @@
       <c r="E7" s="6" t="n"/>
       <c r="F7" s="6" t="n"/>
       <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>FIT
+Siddhartha Kusuma
+38% pred | 0% hist
+[CONSIDER]</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="52" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
@@ -1362,12 +1362,12 @@
 [PINNED]</t>
         </is>
       </c>
-      <c r="H8" s="10" t="inlineStr">
-        <is>
-          <t>Recovery
-Shruti Suresh
-38% pred | 0% hist
-[DROP]</t>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Barre 57
+Shruti Kulkarni
+52% pred | 0% hist
+[PINNED]</t>
         </is>
       </c>
     </row>
@@ -1403,7 +1403,7 @@
       <c r="D10" s="6" t="n"/>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>FIT
+          <t>Back Body Blaze Express
 Shruti Kulkarni
 38% pred | 0% hist
 [DROP]</t>
@@ -1421,22 +1421,57 @@
       <c r="H10" s="6" t="n"/>
     </row>
     <row r="11" ht="52" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>17:15</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="n"/>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="n"/>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>FIT
+Shruti Kulkarni
+38% pred | 0% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Mat 57
+Shruti Kulkarni
+50% pred | 50% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Mat 57
+Shruti Kulkarni
+50% pred | 50% hist
+[PROTECT]</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Mat 57
+Shruti Kulkarni
+38% pred | 0% hist
+[PROTECT]</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>Cardio Barre
-Siddhartha Kusuma
-19% pred | 19% hist
-[CONSIDER]</t>
+Shruti Kulkarni
+38% pred | 0% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>Mat 57
+Pushyank Nahar
+38% pred | 0% hist
+[PROTECT]</t>
         </is>
       </c>
       <c r="H11" s="6" t="n"/>
@@ -1444,55 +1479,55 @@
     <row r="12" ht="52" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Mat 57
-Shruti Kulkarni
-38% pred | 0% hist
-[PROTECT]</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>Mat 57
-Shruti Kulkarni
-50% pred | 50% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>Mat 57
-Pushyank Nahar
-43% pred | 43% hist
-[PROTECT]</t>
-        </is>
-      </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t>Mat 57
-Shruti Kulkarni
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Barre 57
+Chaitanya Nahar
+19% pred | 19% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Barre 57
+Shruti Suresh
+38% pred | 0% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Barre 57
+Siddhartha Kusuma
+31% pred | 31% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Barre 57
+Shruti Suresh
 38% pred | 0% hist
 [CONSIDER]</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
+          <t>FIT
+Pushyank Nahar
+38% pred | 0% hist
+[PROTECT]</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
           <t>Cardio Barre
-Shruti Kulkarni
-38% pred | 0% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="G12" s="9" t="inlineStr">
-        <is>
-          <t>Mat 57
-Pushyank Nahar
-38% pred | 0% hist
-[PROTECT]</t>
+Chaitanya Nahar
+38% pred | 0% hist
+[CONSIDER]</t>
         </is>
       </c>
       <c r="H12" s="6" t="n"/>
@@ -1500,53 +1535,53 @@
     <row r="13" ht="52" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>18:15</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Mat 57
+Shruti Kulkarni
+38% pred | 0% hist
+[PROTECT]</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Recovery
+Shruti Kulkarni
+38% pred | 0% hist
+[PROTECT]</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Back Body Blaze
+Shruti Kulkarni
+38% pred | 0% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>FIT
+Shruti Kulkarni
+38% pred | 0% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>Cardio Barre
-Siddhartha Kusuma
-38% pred | 0% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Barre 57
-Shruti Suresh
-38% pred | 0% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Barre 57
-Siddhartha Kusuma
-31% pred | 31% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Barre 57
-Shruti Suresh
-38% pred | 0% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="F13" s="9" t="inlineStr">
-        <is>
-          <t>Mat 57
-Pushyank Nahar
-38% pred | 0% hist
-[PROTECT]</t>
+Pushyank Nahar
+26% pred | 26% hist
+[CONSIDER]</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
           <t>Recovery
-Shruti Kulkarni
+Pushyank Nahar
 38% pred | 0% hist
 [PROTECT]</t>
         </is>
@@ -1556,25 +1591,11 @@
     <row r="14" ht="52" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>19:15</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>Recovery
-Shruti Kulkarni
-10% pred | 10% hist
-[PROTECT]</t>
-        </is>
-      </c>
-      <c r="C14" s="10" t="inlineStr">
-        <is>
-          <t>Recovery
-Shruti Kulkarni
-38% pred | 0% hist
-[PROTECT]</t>
-        </is>
-      </c>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
       <c r="D14" s="5" t="inlineStr">
         <is>
           <t>FIT
@@ -1583,45 +1604,10 @@
 [PROTECT]</t>
         </is>
       </c>
-      <c r="E14" s="10" t="inlineStr">
-        <is>
-          <t>Recovery
-Shruti Kulkarni
-38% pred | 0% hist
-[PROTECT]</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>Cardio Barre
-Pushyank Nahar
-26% pred | 26% hist
-[CONSIDER]</t>
-        </is>
-      </c>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="n"/>
       <c r="H14" s="6" t="n"/>
-    </row>
-    <row r="15" ht="52" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>19:30</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="n"/>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Back Body Blaze
-Shruti Kulkarni
-38% pred | 0% hist
-[PROTECT]</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="n"/>
-      <c r="G15" s="6" t="n"/>
-      <c r="H15" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1637,7 +1623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1758,9 +1744,9 @@
       <c r="C4" s="6" t="n"/>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Barre 57
-Siddhartha Kusuma
-0% pred | 0% hist
+          <t>Cardio Barre
+Shruti Kulkarni
+38% pred | 0% hist
 [CONSIDER]</t>
         </is>
       </c>
@@ -1863,8 +1849,8 @@
       <c r="C7" s="6" t="n"/>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Barre 57
-Siddhartha Kusuma
+          <t>Cardio Barre Plus
+Pushyank Nahar
 38% pred | 0% hist
 [CONSIDER]</t>
         </is>
@@ -1872,7 +1858,14 @@
       <c r="E7" s="6" t="n"/>
       <c r="F7" s="6" t="n"/>
       <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>FIT
+Siddhartha Kusuma
+38% pred | 0% hist
+[CONSIDER]</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="52" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
@@ -1914,12 +1907,12 @@
 [PINNED]</t>
         </is>
       </c>
-      <c r="H8" s="10" t="inlineStr">
-        <is>
-          <t>Recovery
-Shruti Suresh
-38% pred | 0% hist
-[DROP]</t>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Barre 57
+Shruti Kulkarni
+52% pred | 0% hist
+[PINNED]</t>
         </is>
       </c>
     </row>
@@ -1955,7 +1948,7 @@
       <c r="D10" s="6" t="n"/>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>FIT
+          <t>Back Body Blaze Express
 Shruti Kulkarni
 38% pred | 0% hist
 [DROP]</t>
@@ -1973,22 +1966,57 @@
       <c r="H10" s="6" t="n"/>
     </row>
     <row r="11" ht="52" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>17:15</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="n"/>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="n"/>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>FIT
+Shruti Kulkarni
+38% pred | 0% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Mat 57
+Shruti Kulkarni
+50% pred | 50% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Mat 57
+Shruti Kulkarni
+50% pred | 50% hist
+[PROTECT]</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Mat 57
+Shruti Kulkarni
+38% pred | 0% hist
+[PROTECT]</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>Cardio Barre
-Siddhartha Kusuma
-19% pred | 19% hist
-[CONSIDER]</t>
+Shruti Kulkarni
+38% pred | 0% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>Mat 57
+Pushyank Nahar
+38% pred | 0% hist
+[PROTECT]</t>
         </is>
       </c>
       <c r="H11" s="6" t="n"/>
@@ -1996,55 +2024,55 @@
     <row r="12" ht="52" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Mat 57
-Shruti Kulkarni
-38% pred | 0% hist
-[PROTECT]</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>Mat 57
-Shruti Kulkarni
-50% pred | 50% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>Mat 57
-Pushyank Nahar
-43% pred | 43% hist
-[PROTECT]</t>
-        </is>
-      </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t>Mat 57
-Shruti Kulkarni
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Barre 57
+Chaitanya Nahar
+19% pred | 19% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Barre 57
+Shruti Suresh
+38% pred | 0% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Barre 57
+Siddhartha Kusuma
+31% pred | 31% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Barre 57
+Shruti Suresh
 38% pred | 0% hist
 [CONSIDER]</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
+          <t>FIT
+Pushyank Nahar
+38% pred | 0% hist
+[PROTECT]</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
           <t>Cardio Barre
-Shruti Kulkarni
-38% pred | 0% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="G12" s="9" t="inlineStr">
-        <is>
-          <t>Mat 57
-Pushyank Nahar
-38% pred | 0% hist
-[PROTECT]</t>
+Chaitanya Nahar
+38% pred | 0% hist
+[CONSIDER]</t>
         </is>
       </c>
       <c r="H12" s="6" t="n"/>
@@ -2052,53 +2080,53 @@
     <row r="13" ht="52" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>18:15</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Mat 57
+Shruti Kulkarni
+38% pred | 0% hist
+[PROTECT]</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Recovery
+Shruti Kulkarni
+38% pred | 0% hist
+[PROTECT]</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Back Body Blaze
+Shruti Kulkarni
+38% pred | 0% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>FIT
+Shruti Kulkarni
+38% pred | 0% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>Cardio Barre
-Siddhartha Kusuma
-38% pred | 0% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Barre 57
-Shruti Suresh
-38% pred | 0% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Barre 57
-Siddhartha Kusuma
-31% pred | 31% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Barre 57
-Shruti Suresh
-38% pred | 0% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="F13" s="9" t="inlineStr">
-        <is>
-          <t>Mat 57
-Pushyank Nahar
-38% pred | 0% hist
-[PROTECT]</t>
+Pushyank Nahar
+26% pred | 26% hist
+[CONSIDER]</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
           <t>Recovery
-Shruti Kulkarni
+Pushyank Nahar
 38% pred | 0% hist
 [PROTECT]</t>
         </is>
@@ -2108,25 +2136,11 @@
     <row r="14" ht="52" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>19:15</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>Recovery
-Shruti Kulkarni
-10% pred | 10% hist
-[PROTECT]</t>
-        </is>
-      </c>
-      <c r="C14" s="10" t="inlineStr">
-        <is>
-          <t>Recovery
-Shruti Kulkarni
-38% pred | 0% hist
-[PROTECT]</t>
-        </is>
-      </c>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
       <c r="D14" s="5" t="inlineStr">
         <is>
           <t>FIT
@@ -2135,45 +2149,10 @@
 [PROTECT]</t>
         </is>
       </c>
-      <c r="E14" s="10" t="inlineStr">
-        <is>
-          <t>Recovery
-Shruti Kulkarni
-38% pred | 0% hist
-[PROTECT]</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>Cardio Barre
-Pushyank Nahar
-26% pred | 26% hist
-[CONSIDER]</t>
-        </is>
-      </c>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="n"/>
       <c r="H14" s="6" t="n"/>
-    </row>
-    <row r="15" ht="52" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>19:30</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="n"/>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Back Body Blaze
-Shruti Kulkarni
-38% pred | 0% hist
-[PROTECT]</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="n"/>
-      <c r="G15" s="6" t="n"/>
-      <c r="H15" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>